<commit_message>
run experiments of metaheuristic
</commit_message>
<xml_diff>
--- a/code/resultados/Exp_alpha0.1_NWJSSP_OADG_NEH(MS+ELS+SA).xlsx
+++ b/code/resultados/Exp_alpha0.1_NWJSSP_OADG_NEH(MS+ELS+SA).xlsx
@@ -1,39 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oscar\Desktop\University\Heuristica\Heuristica-Trabajo-3\code\resultados\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A836AE03-2B9A-4D20-8636-FB1A14123FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ft06" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ft06r" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ft10" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ft10r" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ft20" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ft20r" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ft06" sheetId="1" r:id="rId1"/>
+    <sheet name="ft06r" sheetId="2" r:id="rId2"/>
+    <sheet name="ft10" sheetId="3" r:id="rId3"/>
+    <sheet name="ft10r" sheetId="4" r:id="rId4"/>
+    <sheet name="ft20" sheetId="5" r:id="rId5"/>
+    <sheet name="ft20r" sheetId="6" r:id="rId6"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -52,80 +56,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -413,39 +358,35 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1">
         <v>308</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1">
         <v>8149</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>17</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>13</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>40</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>40</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>1</v>
       </c>
     </row>
@@ -455,39 +396,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1">
         <v>321</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1">
         <v>1881</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>16</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>18</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>39</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>3</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>48</v>
       </c>
     </row>
@@ -497,51 +434,47 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1">
         <v>9814</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1">
         <v>163501</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>486</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>197</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>925</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>725</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>65</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>366</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>209</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2">
         <v>562</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>1170</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>0</v>
       </c>
     </row>
@@ -551,51 +484,47 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1">
         <v>10210</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1">
         <v>73205</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>287</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>935</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>1256</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>560</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>166</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>9</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2">
         <v>766</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>627</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>495</v>
       </c>
     </row>
@@ -605,81 +534,77 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:T2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A1">
         <v>17598</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1">
         <v>220465</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>167</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>1400</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>681</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>1014</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>344</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>45</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2">
         <v>119</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>910</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>480</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2">
         <v>247</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2">
         <v>254</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2">
         <v>1260</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2">
         <v>901</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2">
         <v>877</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2">
         <v>392</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2">
         <v>1223</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R2">
         <v>1545</v>
       </c>
-      <c r="S2" t="n">
+      <c r="S2">
         <v>607</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T2">
         <v>23</v>
       </c>
     </row>
@@ -689,99 +614,77 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:T2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A1">
         <v>18268</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1">
         <v>238226</v>
       </c>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
-      <c r="K1" t="inlineStr"/>
-      <c r="L1" t="inlineStr"/>
-      <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
-      <c r="O1" t="inlineStr"/>
-      <c r="P1" t="inlineStr"/>
-      <c r="Q1" t="inlineStr"/>
-      <c r="R1" t="inlineStr"/>
-      <c r="S1" t="inlineStr"/>
-      <c r="T1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>7</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>1365</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>689</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>573</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>259</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>499</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2">
         <v>413</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>1476</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>993</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2">
         <v>802</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2">
         <v>444</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2">
         <v>824</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2">
         <v>1139</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2">
         <v>1603</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2">
         <v>300</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2">
         <v>606</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R2">
         <v>992</v>
       </c>
-      <c r="S2" t="n">
+      <c r="S2">
         <v>101</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T2">
         <v>74</v>
       </c>
     </row>

</xml_diff>